<commit_message>
setting parameters for retriever, prompt, openai(temperature) to control the experiment about performance of chatbot RAG system
</commit_message>
<xml_diff>
--- a/RAG_qa.xlsx
+++ b/RAG_qa.xlsx
@@ -1,21 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hyeongdohun/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hyeongdohun/Documents/2024_proj_openai/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03DEF482-9CAD-544B-BD17-5A86E2F9BABE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FDEE48C-F68F-CE4B-BFE6-E0AC892904BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -6281,7 +6294,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D698"/>
+  <dimension ref="A1:D699"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="63.83203125" customWidth="1"/>
@@ -16062,6 +16075,16 @@
         <v>0.33333333333333331</v>
       </c>
     </row>
+    <row r="699" spans="1:4">
+      <c r="C699">
+        <f>AVERAGE(C2:C676)</f>
+        <v>0.73200255488356059</v>
+      </c>
+      <c r="D699">
+        <f>AVERAGE(D2:D676)</f>
+        <v>0.79013648080314713</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>